<commit_message>
Audit final benchmark scoring repairs
</commit_message>
<xml_diff>
--- a/results/qwen25vl3b_7b_answer_grpo_selected25_temp06_3seed_mean_std.xlsx
+++ b/results/qwen25vl3b_7b_answer_grpo_selected25_temp06_3seed_mean_std.xlsx
@@ -2602,7 +2602,7 @@
         <v>45.1777</v>
       </c>
       <c r="G32" t="n">
-        <v>3.934</v>
+        <v>3.934000000000005</v>
       </c>
       <c r="H32" t="n">
         <v>1.5229</v>
@@ -2633,7 +2633,7 @@
         <v>6.5989</v>
       </c>
       <c r="H33" t="n">
-        <v>3.0457</v>
+        <v>3.045699999999997</v>
       </c>
     </row>
     <row r="34">
@@ -2658,10 +2658,10 @@
         <v>47.335</v>
       </c>
       <c r="G34" t="n">
-        <v>5.9644</v>
+        <v>5.964400000000005</v>
       </c>
       <c r="H34" t="n">
-        <v>3.1726</v>
+        <v>3.172600000000003</v>
       </c>
     </row>
     <row r="35">
@@ -3935,7 +3935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4108,6 +4108,23 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>mathverse_judgement_repair</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MathVerse local Qwen3-32B judge outputs of the form `Judgement: 1` are counted as correct.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>No generation or judge rerun.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>